<commit_message>
Use local copy of emmo in excelparsertest
</commit_message>
<xml_diff>
--- a/tests/test_excelparser/onto.xlsx
+++ b/tests/test_excelparser/onto.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\flb\projects\Team4.0\EMMOntoPy\tests\test_excelparser\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\flb\projects\interoperability_tools\EMMOntoPy\tests\test_excelparser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F62E00-332A-4644-BCFE-58C676F44153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F61E52-537E-4415-9FD3-6715048151FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-48090" yWindow="-6765" windowWidth="38700" windowHeight="15345" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-48915" yWindow="-3795" windowWidth="34470" windowHeight="17640" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -542,7 +542,7 @@
     <t>Check adding more than one annotation</t>
   </si>
   <si>
-    <t>https://w3id.org/emmo/inferred</t>
+    <t>https://raw.githubusercontent.com/emmo-repo/EMMOntoPy/refs/heads/master/tests/testonto/emmo/emmo-squashed.ttl</t>
   </si>
 </sst>
 </file>
@@ -1294,11 +1294,8 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{33CC3B70-5CD5-4594-B662-DF452B3A2B7A}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Exceltool fails emmoupdate (#923)
</commit_message>
<xml_diff>
--- a/tests/test_excelparser/onto.xlsx
+++ b/tests/test_excelparser/onto.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\flb\projects\Team4.0\EMMOntoPy\tests\test_excelparser\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\flb\projects\interoperability_tools\EMMOntoPy\tests\test_excelparser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F62E00-332A-4644-BCFE-58C676F44153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F61E52-537E-4415-9FD3-6715048151FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-48090" yWindow="-6765" windowWidth="38700" windowHeight="15345" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-48915" yWindow="-3795" windowWidth="34470" windowHeight="17640" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -542,7 +542,7 @@
     <t>Check adding more than one annotation</t>
   </si>
   <si>
-    <t>https://w3id.org/emmo/inferred</t>
+    <t>https://raw.githubusercontent.com/emmo-repo/EMMOntoPy/refs/heads/master/tests/testonto/emmo/emmo-squashed.ttl</t>
   </si>
 </sst>
 </file>
@@ -1294,11 +1294,8 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{33CC3B70-5CD5-4594-B662-DF452B3A2B7A}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>